<commit_message>
Move Sheet formulas to generated Apps Script setup (xlsx import drops Sheets-only functions)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BTVXsqWJ6LyrW5pT3WwZLR
</commit_message>
<xml_diff>
--- a/golden-goose-opening/sheet/GG_Opening_Action_Log.xlsx
+++ b/golden-goose-opening/sheet/GG_Opening_Action_Log.xlsx
@@ -686,9 +686,10 @@
           <t>Latest Update Date</t>
         </is>
       </c>
-      <c r="Q1" s="2">
-        <f>{"Update History";BYROW(A2:A,LAMBDA(id,IF(id="","",IFERROR(TEXTJOIN(CHAR(10),TRUE,SORT(FILTER(TEXT(TASK_HISTORY!B2:B,"dd/mm/yy")&amp;" – "&amp;IF(TASK_HISTORY!F2:F="Decision","DECISION: ","")&amp;TASK_HISTORY!J2:J,TASK_HISTORY!D2:D=id,TASK_HISTORY!J2:J&lt;&gt;""),FILTER(TASK_HISTORY!B2:B,TASK_HISTORY!D2:D=id,TASK_HISTORY!J2:J&lt;&gt;""),FALSE,FILTER(TASK_HISTORY!C2:C,TASK_HISTORY!D2:D=id,TASK_HISTORY!J2:J&lt;&gt;""),FALSE)),""))))}</f>
-        <v/>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Update History</t>
+        </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
@@ -705,9 +706,10 @@
           <t>Critical for Opening</t>
         </is>
       </c>
-      <c r="U1" s="2">
-        <f>{"Check";ARRAYFORMULA(IF((A2:A="")*(F2:F=""),"",REGEXREPLACE(REGEXREPLACE(IF((A2:A="")*(F2:F&lt;&gt;""),"⛔ Task ID mancante · ","")&amp;IF((A2:A&lt;&gt;"")*(COUNTIF(A2:A,A2:A)&gt;1),"⛔ Task ID duplicato · ","")&amp;IF((A2:A&lt;&gt;"")*(IFERROR((MID(A2:A,LEN(A2:A)-3,1)&lt;&gt;"-")+ISERROR(VALUE(RIGHT(A2:A,3))),1)&gt;0),"⛔ Formato Task ID · ","")&amp;IF(((B2:B="")+(C2:C="")+(D2:D="")+(F2:F="")+(H2:H="")+(I2:I="")&gt;0),"⛔ Campi obbligatori mancanti · ","")&amp;IF((B2:B&lt;&gt;"")*(C2:C&lt;&gt;"")*(COUNTIFS(OPENINGS!B2:B,B2:B,OPENINGS!C2:C,C2:C)=0),"⛔ Type + Location inesistente · ","")&amp;IF((A2:A&lt;&gt;"")*(COUNTIFS(OPENINGS!A2:A,IFERROR(LEFT(A2:A,LEN(A2:A)-4),"#"),OPENINGS!B2:B,B2:B,OPENINGS!C2:C,C2:C)=0),"⛔ Prefisso ID ≠ Opening · ","")&amp;IF((D2:D&lt;&gt;"")*IF(E2:E="",COUNTIF(AREAS!A2:A,D2:D)=0,COUNTIFS(AREAS!A2:A,D2:D,AREAS!B2:B,E2:E)=0),"⛔ Macro / Sub Area non valida · ","")&amp;IF((H2:H&lt;&gt;"")*(COUNTIF(LISTS!A2:A,H2:H)=0),"⛔ Status non valido · ","")&amp;IF((I2:I&lt;&gt;"")*(COUNTIF(LISTS!B2:B,I2:I)=0),"⛔ Progress non valido · ","")&amp;IF(((J2:J&lt;&gt;"")*(COUNTIF(OWNERS!A2:A,J2:J)=0)+(K2:K&lt;&gt;"")*(COUNTIF(OWNERS!A2:A,K2:K)=0)+(L2:L&lt;&gt;"")*(COUNTIF(OWNERS!A2:A,L2:L)=0)&gt;0),"⛔ Owner non in OWNERS · ","")&amp;IF(((M2:M&lt;&gt;"")*NOT(ISNUMBER(M2:M))+(N2:N&lt;&gt;"")*NOT(ISNUMBER(N2:N))+(P2:P&lt;&gt;"")*NOT(ISNUMBER(P2:P))&gt;0),"⛔ Data non valida · ","")&amp;IF((J2:J="")*((K2:K&lt;&gt;"")+(L2:L&lt;&gt;"")&gt;0),"⛔ Owner 2/3 senza Owner 1 · ","")&amp;IF((H2:H&lt;&gt;"Completed")*(H2:H&lt;&gt;"N/A")*(J2:J=""),"⚠ Owner 1 mancante · ","")&amp;IF((H2:H&lt;&gt;"Completed")*(H2:H&lt;&gt;"N/A")*(N2:N=""),"⚠ Due Date mancante · ","")&amp;IF((H2:H="Completed")*(I2:I&lt;&gt;100),"⚠ Completed con Progress &lt; 100% · ","")&amp;IF((I2:I=100)*(H2:H&lt;&gt;"Completed"),"⚠ 100% ma non Completed · ","")&amp;IF(((H2:H="Blocked")+(S2:S=TRUE)&gt;0)*(R2:R=""),"⚠ Blocker / Decision vuoto · ","")&amp;IF((H2:H="N/A")*(O2:O=""),"⚠ N/A senza motivazione · ","")&amp;IF((O2:O&lt;&gt;"")*(P2:P=""),"⚠ Latest Update senza data · ","")&amp;IF((IFERROR((M2:M&gt;TODAY())+(P2:P&gt;TODAY()),0)&gt;0),"⚠ Data futura · ","")&amp;IF((M2:M&lt;&gt;"")*(N2:N&lt;&gt;"")*(M2:M&gt;N2:N),"⚠ Open Date dopo Due Date · ","")&amp;IF((T2:T=TRUE)*(H2:H&lt;&gt;"Completed")*(H2:H&lt;&gt;"N/A")*(N2:N&lt;&gt;"")*(N2:N&gt;SUMIFS(OPENINGS!J2:J,OPENINGS!B2:B,B2:B,OPENINGS!C2:C,C2:C)),"⚠ Critico con scadenza oltre l'apertura · ","")&amp;IF(((J2:J&lt;&gt;"")*((J2:J=K2:K)+(J2:J=L2:L))+(K2:K&lt;&gt;"")*(K2:K=L2:L)&gt;0),"⚠ Owner ripetuto · ","")&amp;"|"," · \|$",""),"^\|$","OK")))}</f>
-        <v/>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
       </c>
       <c r="V1" s="2" t="inlineStr">
         <is>
@@ -3168,9 +3170,10 @@
           <t>Verification</t>
         </is>
       </c>
-      <c r="O1" s="2">
-        <f>{"Check";ARRAYFORMULA(IF(D2:D="","",IF(COUNTIF(ACTION_LOG!A2:A,D2:D)=0,"⛔ Task ID inesistente",IF(B2:B="","⛔ Event Date mancante","OK"))))}</f>
-        <v/>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
       </c>
     </row>
     <row r="2">
@@ -5005,41 +5008,50 @@
           <t>Related Opening</t>
         </is>
       </c>
-      <c r="I1" s="2">
-        <f>{"Baseline Opening Date";ARRAYFORMULA(IF(A2:A="","",IFERROR(VLOOKUP(A2:A,FILTER(OPENING_DATE_HISTORY!B2:E,OPENING_DATE_HISTORY!C2:C="Baseline"),4,FALSE),"")))}</f>
-        <v/>
-      </c>
-      <c r="J1" s="2">
-        <f>{"Current Opening Date";ARRAYFORMULA(IF(A2:A="","",IFERROR(VLOOKUP(A2:A,SORT(FILTER(OPENING_DATE_HISTORY!B2:E,OPENING_DATE_HISTORY!B2:B&lt;&gt;""),FILTER(OPENING_DATE_HISTORY!D2:D,OPENING_DATE_HISTORY!B2:B&lt;&gt;""),FALSE,FILTER(ROW(OPENING_DATE_HISTORY!B2:B),OPENING_DATE_HISTORY!B2:B&lt;&gt;""),FALSE),4,FALSE),"")))}</f>
-        <v/>
-      </c>
-      <c r="K1" s="2">
-        <f>{"Delay (wd)";ARRAYFORMULA(IF((I2:I="")+(J2:J="")&gt;0,"",IF(J2:J&gt;=I2:I,NETWORKDAYS(I2:I,J2:J)-1,-(NETWORKDAYS(J2:J,I2:I)-1))))}</f>
-        <v/>
-      </c>
-      <c r="L1" s="2">
-        <f>{"Postponements";ARRAYFORMULA(IF(A2:A="","",COUNTIFS(OPENING_DATE_HISTORY!B2:B,A2:A,OPENING_DATE_HISTORY!C2:C,"Change")))}</f>
-        <v/>
-      </c>
-      <c r="M1" s="2">
-        <f>{"Days Elapsed (wd)";ARRAYFORMULA(IF((F2:F="")+(J2:J="")&gt;0,"",IF(G2:G="Opened",NETWORKDAYS(F2:F,J2:J),NETWORKDAYS(F2:F,TODAY()))))}</f>
-        <v/>
-      </c>
-      <c r="N1" s="2">
-        <f>{"Planned Duration (wd)";ARRAYFORMULA(IF((F2:F="")+(J2:J="")&gt;0,"",NETWORKDAYS(F2:F,J2:J)))}</f>
-        <v/>
-      </c>
-      <c r="O1" s="2">
-        <f>{"Days Remaining (wd)";ARRAYFORMULA(IF(J2:J="","",IF(G2:G="Opened",0,IF(J2:J&gt;=TODAY(),NETWORKDAYS(TODAY(),J2:J)-1,-(NETWORKDAYS(J2:J,TODAY())-1)))))}</f>
-        <v/>
-      </c>
-      <c r="P1" s="2">
-        <f>{"Next Task ID";ARRAYFORMULA(IF(A2:A="","",A2:A&amp;"-"&amp;TEXT(COUNTIF(ACTION_LOG!A2:A,A2:A&amp;"-???")+1,"000")))}</f>
-        <v/>
-      </c>
-      <c r="Q1" s="2">
-        <f>{"Check";ARRAYFORMULA(IF(A2:A="","",IF(COUNTIF(A2:A,A2:A)&gt;1,"⛔ Codice duplicato",IF(COUNTIFS(B2:B,B2:B,C2:C,C2:C)&gt;1,"⛔ Type + Location duplicato",IF(COUNTIFS(OPENING_DATE_HISTORY!B2:B,A2:A,OPENING_DATE_HISTORY!C2:C,"Baseline")&lt;&gt;1,"⛔ Serve una (sola) riga Baseline","OK")))))}</f>
-        <v/>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Baseline Opening Date</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Current Opening Date</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Delay (wd)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Postponements</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Days Elapsed (wd)</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Planned Duration (wd)</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Days Remaining (wd)</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Next Task ID</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
       </c>
     </row>
     <row r="2">
@@ -5875,13 +5887,15 @@
           <t>New Opening Date</t>
         </is>
       </c>
-      <c r="F1" s="2">
-        <f>{"Previous Date";BYROW(B2:E,LAMBDA(r,IF(INDEX(r,1,2)&lt;&gt;"Change","",IFERROR(SUMIFS(E2:E,B2:B,INDEX(r,1,1),D2:D,MAXIFS(D2:D,B2:B,INDEX(r,1,1),D2:D,"&lt;"&amp;INDEX(r,1,3))),""))))}</f>
-        <v/>
-      </c>
-      <c r="G1" s="2">
-        <f>{"Shift (wd)";ARRAYFORMULA(IF((C2:C&lt;&gt;"Change")+(F2:F="")&gt;0,"",IF(E2:E&gt;=F2:F,NETWORKDAYS(F2:F,E2:E)-1,-(NETWORKDAYS(E2:E,F2:F)-1))))}</f>
-        <v/>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Previous Date</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Shift (wd)</t>
+        </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
@@ -6795,17 +6809,20 @@
           <t>Run By</t>
         </is>
       </c>
-      <c r="G1" s="2">
-        <f>{"Changes";ARRAYFORMULA(IF(A2:A="","",COUNTIF(TASK_HISTORY!M2:M,A2:A)))}</f>
-        <v/>
-      </c>
-      <c r="H1" s="2">
-        <f>{"Verified";ARRAYFORMULA(IF(A2:A="","",COUNTIFS(TASK_HISTORY!M2:M,A2:A,TASK_HISTORY!N2:N,"Verified")))}</f>
-        <v/>
-      </c>
-      <c r="I1" s="2">
-        <f>{"Mismatches";ARRAYFORMULA(IF(A2:A="","",COUNTIFS(TASK_HISTORY!M2:M,A2:A,TASK_HISTORY!N2:N,"Mismatch")))}</f>
-        <v/>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Changes</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Mismatches</t>
+        </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
@@ -7642,18 +7659,6 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="L2">
-        <f>SORT(UNIQUE(FILTER(OPENINGS!C2:C,OPENINGS!C2:C&lt;&gt;"")))</f>
-        <v/>
-      </c>
-      <c r="M2">
-        <f>UNIQUE(FILTER(AREAS!A2:A,AREAS!A2:A&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="N2">
-        <f>FILTER(AREAS!B2:B,AREAS!B2:B&lt;&gt;"")</f>
-        <v/>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>Golden Goose</t>

</xml_diff>